<commit_message>
Updated artwork Added as-built rev 1 PCB
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamster\Documents\Development\Badges\dczia\mk9-badge\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{210BEA28-4839-403E-A04F-56A0E9998728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3AE1892-83DF-4DFD-8F58-6AE0A8227181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="27410" windowHeight="17230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39740" yWindow="1830" windowWidth="27410" windowHeight="17230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="111">
   <si>
     <t>Part Number</t>
   </si>
@@ -105,15 +104,6 @@
     <t>https://cdn-shop.adafruit.com/datasheets/WS2812B.pdf</t>
   </si>
   <si>
-    <t>Micro_SD_Card_SPI</t>
-  </si>
-  <si>
-    <t>lib_fp:MicroSD-Socket-Seeed-320090008</t>
-  </si>
-  <si>
-    <t>https://statics3.seeedstudio.com/images/opl/datasheet/320090008.pdf</t>
-  </si>
-  <si>
     <t>USB-C</t>
   </si>
   <si>
@@ -177,18 +167,12 @@
     <t>Cost Each</t>
   </si>
   <si>
-    <t>Cost per Badge</t>
-  </si>
-  <si>
     <t>Distributor</t>
   </si>
   <si>
     <t>Distributor Part</t>
   </si>
   <si>
-    <t>Qty Needed</t>
-  </si>
-  <si>
     <t>Qty Ordered</t>
   </si>
   <si>
@@ -264,9 +248,6 @@
     <t>https://goodarksemi.com/docs/datasheets/mems/GSDA213_SDS.pdf</t>
   </si>
   <si>
-    <t>Total Parts</t>
-  </si>
-  <si>
     <t>PCB</t>
   </si>
   <si>
@@ -291,9 +272,6 @@
     <t>https://www.winbond.com/resource-files/W25Q128JV%20RevI%2008232021%20Plus.pdf</t>
   </si>
   <si>
-    <t>Badge run</t>
-  </si>
-  <si>
     <t>120</t>
   </si>
   <si>
@@ -385,6 +363,9 @@
   </si>
   <si>
     <t>https://www.onsemi.com/pdf/datasheet/ncp115-d.pdf</t>
+  </si>
+  <si>
+    <t>Badge Run, units</t>
   </si>
 </sst>
 </file>
@@ -785,7 +766,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P983"/>
+  <dimension ref="A1:N982"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7265625" customWidth="1"/>
@@ -797,21 +778,19 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="9.6328125" style="5" customWidth="1"/>
     <col min="9" max="10" width="7.1796875" customWidth="1"/>
-    <col min="11" max="11" width="7.453125" style="5" customWidth="1"/>
-    <col min="12" max="12" width="7.54296875" customWidth="1"/>
-    <col min="13" max="13" width="7.36328125" customWidth="1"/>
-    <col min="14" max="14" width="14.6328125" customWidth="1"/>
-    <col min="15" max="15" width="8.453125" customWidth="1"/>
-    <col min="16" max="16" width="10.453125" customWidth="1"/>
-    <col min="17" max="17" width="12.90625" customWidth="1"/>
+    <col min="11" max="11" width="7.36328125" customWidth="1"/>
+    <col min="12" max="12" width="14.6328125" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" customWidth="1"/>
+    <col min="14" max="14" width="10.453125" customWidth="1"/>
+    <col min="15" max="15" width="12.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="16" customFormat="1" ht="35.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="16" customFormat="1" ht="35.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>13</v>
@@ -823,10 +802,10 @@
         <v>0</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H1" s="16" t="s">
         <v>15</v>
@@ -835,30 +814,24 @@
         <v>16</v>
       </c>
       <c r="J1" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="15" t="s">
-        <v>47</v>
-      </c>
       <c r="L1" s="15" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -876,26 +849,18 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="K2">
-        <f>I2*J2</f>
-        <v>5.6000000000000001E-2</v>
-      </c>
-      <c r="L2" s="8">
-        <f>I2*$K$43</f>
-        <v>1680</v>
-      </c>
-      <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2">
+      <c r="L2">
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>18</v>
@@ -912,28 +877,20 @@
       <c r="J3" s="1">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="K3">
-        <f t="shared" ref="K3:K39" si="0">I3*J3</f>
-        <v>1.6E-2</v>
-      </c>
-      <c r="L3" s="8">
-        <f>I3*$K$43</f>
-        <v>480</v>
-      </c>
-      <c r="M3" s="1">
+      <c r="K3" s="1">
         <v>0</v>
       </c>
-      <c r="N3" s="1">
+      <c r="L3" s="1">
         <v>3500</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>9</v>
@@ -951,21 +908,13 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="K4">
-        <f t="shared" si="0"/>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="L4" s="8">
-        <f>I4*$K$43</f>
-        <v>240</v>
-      </c>
-      <c r="M4">
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="L4">
         <v>3500</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="D5" s="8"/>
@@ -973,27 +922,25 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="K5"/>
-      <c r="L5" s="8"/>
-    </row>
-    <row r="6" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="I6" s="1">
         <v>2</v>
@@ -1001,27 +948,19 @@
       <c r="J6" s="1">
         <v>0.11</v>
       </c>
-      <c r="K6">
-        <f t="shared" si="0"/>
-        <v>0.22</v>
-      </c>
-      <c r="L6" s="8">
-        <f>I6*$K$43</f>
-        <v>240</v>
-      </c>
-      <c r="M6" s="1">
+      <c r="K6" s="1">
         <v>0</v>
       </c>
-      <c r="N6" s="1">
+      <c r="L6" s="1">
         <v>2500</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>20</v>
@@ -1033,7 +972,7 @@
         <v>4</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>22</v>
@@ -1044,27 +983,19 @@
       <c r="J7" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="K7">
-        <f t="shared" si="0"/>
-        <v>0.63000000000000012</v>
-      </c>
-      <c r="L7" s="8">
-        <f>I7*$K$43</f>
-        <v>1080</v>
-      </c>
-      <c r="M7" s="1">
+      <c r="K7" s="1">
         <v>0</v>
       </c>
-      <c r="N7" s="1">
+      <c r="L7" s="1">
         <v>2000</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D8" s="6"/>
       <c r="F8" s="1" t="s">
@@ -1077,40 +1008,32 @@
       <c r="J8" s="1">
         <v>0.1</v>
       </c>
-      <c r="K8">
-        <f t="shared" si="0"/>
-        <v>0.60000000000000009</v>
-      </c>
-      <c r="L8" s="8">
-        <f>I8*$K$43</f>
-        <v>720</v>
-      </c>
-      <c r="M8" s="1">
+      <c r="K8" s="1">
         <v>1000</v>
       </c>
-      <c r="N8" s="1">
+      <c r="L8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="I9" s="1">
         <v>0</v>
@@ -1118,25 +1041,18 @@
       <c r="J9" s="1">
         <v>0.38300000000000001</v>
       </c>
-      <c r="K9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L9" s="8">
-        <f>I9*$K$43</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="M9" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="D10" s="6"/>
       <c r="H10" s="6"/>
-      <c r="K10"/>
-      <c r="L10" s="8"/>
-    </row>
-    <row r="11" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="C11" s="1" t="s">
         <v>23</v>
       </c>
@@ -1146,77 +1062,61 @@
       <c r="F11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H11" s="10" t="s">
-        <v>25</v>
+      <c r="G11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>53</v>
       </c>
       <c r="I11" s="1">
         <v>1</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="K11" s="1">
+        <v>150</v>
+      </c>
+      <c r="L11" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E12" s="6"/>
+      <c r="I12" s="6"/>
+    </row>
+    <row r="13" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="K13" s="1">
         <v>0</v>
       </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11" s="8">
-        <f>I11*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="L13" s="1">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="I12" s="1">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0.19</v>
-      </c>
-      <c r="K12">
-        <f>I12*J12</f>
-        <v>0.19</v>
-      </c>
-      <c r="L12" s="8">
-        <f>I12*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M12" s="1">
-        <v>150</v>
-      </c>
-      <c r="N12" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="E13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="L13" s="8"/>
-    </row>
-    <row r="14" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>9</v>
@@ -1230,27 +1130,19 @@
       <c r="J14" s="1">
         <v>1E-3</v>
       </c>
-      <c r="K14">
-        <f t="shared" si="0"/>
-        <v>2E-3</v>
-      </c>
-      <c r="L14" s="8">
-        <f t="shared" ref="L14:L19" si="1">I14*$K$43</f>
-        <v>240</v>
-      </c>
-      <c r="M14" s="1">
+      <c r="K14" s="1">
         <v>0</v>
       </c>
-      <c r="N14" s="1">
+      <c r="L14" s="1">
         <v>4500</v>
       </c>
     </row>
-    <row r="15" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>9</v>
@@ -1264,27 +1156,19 @@
       <c r="J15" s="1">
         <v>1E-3</v>
       </c>
-      <c r="K15">
-        <f t="shared" si="0"/>
-        <v>2E-3</v>
-      </c>
-      <c r="L15" s="8">
-        <f t="shared" si="1"/>
-        <v>240</v>
-      </c>
-      <c r="M15" s="1">
+      <c r="K15" s="1">
         <v>0</v>
       </c>
-      <c r="N15" s="1">
+      <c r="L15" s="1">
         <v>4500</v>
       </c>
     </row>
-    <row r="16" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>9</v>
@@ -1298,27 +1182,19 @@
       <c r="J16" s="1">
         <v>1E-3</v>
       </c>
-      <c r="K16">
-        <f t="shared" si="0"/>
-        <v>2E-3</v>
-      </c>
-      <c r="L16" s="8">
-        <f t="shared" si="1"/>
-        <v>240</v>
-      </c>
-      <c r="M16" s="1">
+      <c r="K16" s="1">
         <v>0</v>
       </c>
-      <c r="N16" s="1">
+      <c r="L16" s="1">
         <v>4500</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>108</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>9</v>
@@ -1327,668 +1203,504 @@
         <v>17</v>
       </c>
       <c r="I17" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="1">
         <v>1E-3</v>
       </c>
-      <c r="K17">
-        <f t="shared" si="0"/>
-        <v>2E-3</v>
-      </c>
-      <c r="L17" s="8">
-        <f t="shared" si="1"/>
-        <v>240</v>
-      </c>
-      <c r="M17" s="1">
+      <c r="K17" s="1">
         <v>0</v>
       </c>
-      <c r="N17" s="1">
+      <c r="L17" s="1">
         <v>4500</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>104</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H18" s="6" t="s">
-        <v>17</v>
-      </c>
+      <c r="H18" s="6"/>
       <c r="I18" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" s="1">
         <v>1E-3</v>
       </c>
-      <c r="K18">
-        <f t="shared" si="0"/>
-        <v>1E-3</v>
-      </c>
-      <c r="L18" s="8">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-      <c r="M18" s="1">
+      <c r="K18" s="19">
+        <v>5000</v>
+      </c>
+      <c r="L18" s="1">
         <v>0</v>
       </c>
-      <c r="N18" s="1">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D19" s="6" t="s">
+    </row>
+    <row r="19" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="I20" s="1">
+        <v>2</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.20204</v>
+      </c>
+      <c r="K20" s="19">
+        <v>300</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" s="1">
+        <v>1</v>
+      </c>
+      <c r="J21" s="13">
+        <v>0.60319999999999996</v>
+      </c>
+      <c r="K21" s="19">
+        <v>150</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="F22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H22" s="10"/>
+      <c r="I22" s="1">
         <v>9</v>
       </c>
-      <c r="H19" s="6"/>
-      <c r="I19" s="1">
+      <c r="J22" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="K22" s="1">
+        <v>1000</v>
+      </c>
+      <c r="L22" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="I24" s="1">
+        <v>1</v>
+      </c>
+      <c r="J24" s="1">
+        <v>6.7699999999999996E-2</v>
+      </c>
+      <c r="K24" s="1">
+        <v>0</v>
+      </c>
+      <c r="L24" s="1">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J19" s="1">
-        <v>1E-3</v>
-      </c>
-      <c r="K19">
-        <f t="shared" si="0"/>
-        <v>2E-3</v>
-      </c>
-      <c r="L19" s="8">
-        <f t="shared" si="1"/>
-        <v>240</v>
-      </c>
-      <c r="M19" s="19">
-        <v>0</v>
-      </c>
-      <c r="N19" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="D20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="K20"/>
-      <c r="L20" s="8"/>
-    </row>
-    <row r="21" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H21" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="I21" s="1">
-        <v>2</v>
-      </c>
-      <c r="J21" s="1">
-        <v>0.20204</v>
-      </c>
-      <c r="K21">
-        <f t="shared" si="0"/>
-        <v>0.40407999999999999</v>
-      </c>
-      <c r="L21" s="8">
-        <f>I21*$K$43</f>
-        <v>240</v>
-      </c>
-      <c r="M21" s="19">
-        <v>0</v>
-      </c>
-      <c r="N21" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="I22" s="1">
-        <v>1</v>
-      </c>
-      <c r="J22" s="13">
-        <v>0.60319999999999996</v>
-      </c>
-      <c r="K22">
-        <f t="shared" si="0"/>
-        <v>0.60319999999999996</v>
-      </c>
-      <c r="L22" s="8">
-        <f>I22*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M22" s="19">
-        <v>0</v>
-      </c>
-      <c r="N22" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D23" s="6"/>
-      <c r="F23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H23" s="10"/>
-      <c r="I23" s="1">
-        <v>9</v>
-      </c>
-      <c r="J23" s="13">
-        <v>0.1</v>
-      </c>
-      <c r="K23">
-        <f t="shared" si="0"/>
-        <v>0.9</v>
-      </c>
-      <c r="L23" s="8">
-        <f>I23*$K$43</f>
-        <v>1080</v>
-      </c>
-      <c r="M23" s="1">
-        <v>1000</v>
-      </c>
-      <c r="N23" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="D24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="K24"/>
-      <c r="L24" s="8"/>
-    </row>
-    <row r="25" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="G25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>116</v>
       </c>
       <c r="I25" s="1">
         <v>1</v>
       </c>
-      <c r="J25" s="1">
-        <v>6.7699999999999996E-2</v>
-      </c>
-      <c r="K25">
-        <f t="shared" si="0"/>
-        <v>6.7699999999999996E-2</v>
-      </c>
-      <c r="L25" s="8">
-        <f>I25*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M25" s="1">
+      <c r="J25" s="12">
+        <v>0.8</v>
+      </c>
+      <c r="K25" s="1">
         <v>0</v>
       </c>
-      <c r="N25" s="1">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="L25" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>52</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D26" s="6"/>
       <c r="F26" s="1" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>40</v>
+        <v>77</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="I26" s="1">
         <v>1</v>
       </c>
-      <c r="J26" s="12">
-        <v>0.8</v>
-      </c>
-      <c r="K26">
-        <f t="shared" si="0"/>
-        <v>0.8</v>
-      </c>
-      <c r="L26" s="8">
-        <f>I26*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M26" s="1">
+      <c r="J26" s="13">
+        <v>2.5155599999999998</v>
+      </c>
+      <c r="K26" s="19">
+        <v>133</v>
+      </c>
+      <c r="L26" s="1">
         <v>0</v>
       </c>
-      <c r="N26" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H27" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D27" s="6"/>
-      <c r="F27" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="I27" s="1">
         <v>1</v>
       </c>
       <c r="J27" s="13">
-        <v>2.5155599999999998</v>
-      </c>
-      <c r="K27">
-        <f t="shared" si="0"/>
-        <v>2.5155599999999998</v>
-      </c>
-      <c r="L27" s="8">
-        <f>I27*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M27" s="19">
+        <v>0.65949999999999998</v>
+      </c>
+      <c r="K27" s="19">
+        <v>150</v>
+      </c>
+      <c r="L27" s="1">
         <v>0</v>
       </c>
-      <c r="N27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="I28" s="1">
-        <v>1</v>
-      </c>
-      <c r="J28" s="13">
-        <v>0.65949999999999998</v>
-      </c>
-      <c r="K28">
-        <f t="shared" si="0"/>
-        <v>0.65949999999999998</v>
-      </c>
-      <c r="L28" s="8">
-        <f>I28*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M28" s="19">
-        <v>0</v>
-      </c>
-      <c r="N28" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="J28" s="13"/>
+    </row>
+    <row r="29" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="D29" s="6"/>
       <c r="H29" s="6"/>
-      <c r="J29" s="13"/>
-      <c r="K29"/>
-      <c r="L29" s="8"/>
-    </row>
-    <row r="30" spans="1:16" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="D30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="J30" s="11"/>
-      <c r="K30"/>
-      <c r="L30" s="8"/>
-    </row>
-    <row r="31" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="J29" s="11"/>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I30">
+        <v>2</v>
+      </c>
+      <c r="J30" s="13"/>
+      <c r="N30" s="1"/>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E31" s="3"/>
+      <c r="N31" s="1"/>
+    </row>
+    <row r="32" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D32" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I31">
-        <v>2</v>
-      </c>
-      <c r="J31" s="13"/>
-      <c r="K31">
-        <f t="shared" si="0"/>
+      <c r="E32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="I32" s="1">
+        <v>1</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0.40849999999999997</v>
+      </c>
+      <c r="K32" s="19">
+        <v>150</v>
+      </c>
+      <c r="L32" s="1">
         <v>0</v>
       </c>
-      <c r="L31" s="8"/>
-      <c r="P31" s="1"/>
-    </row>
-    <row r="32" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E32" s="3"/>
-      <c r="K32"/>
-      <c r="L32" s="8"/>
-      <c r="P32" s="1"/>
-    </row>
-    <row r="33" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="I33" s="1">
-        <v>1</v>
-      </c>
-      <c r="J33" s="1">
-        <v>0.40849999999999997</v>
-      </c>
-      <c r="K33">
-        <f t="shared" si="0"/>
-        <v>0.40849999999999997</v>
-      </c>
-      <c r="L33" s="8">
-        <f>I33*$K$43</f>
-        <v>120</v>
-      </c>
-      <c r="M33" s="19">
-        <v>0</v>
-      </c>
-      <c r="N33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D33" s="6"/>
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="1:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="D34" s="6"/>
       <c r="H34" s="6"/>
-      <c r="K34"/>
-    </row>
-    <row r="35" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C35" s="1" t="s">
+        <v>108</v>
+      </c>
       <c r="D35" s="6"/>
       <c r="H35" s="6"/>
-      <c r="K35"/>
-    </row>
-    <row r="36" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="I35" s="1">
+        <v>9</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="K35" s="1">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="2"/>
       <c r="C36" s="1" t="s">
-        <v>115</v>
+        <v>62</v>
       </c>
       <c r="D36" s="6"/>
       <c r="H36" s="6"/>
       <c r="I36" s="1">
-        <v>9</v>
-      </c>
-      <c r="J36" s="1">
-        <v>0.19</v>
-      </c>
-      <c r="K36">
-        <f t="shared" si="0"/>
-        <v>1.71</v>
-      </c>
-      <c r="L36" s="8">
-        <f>I36*$K$43</f>
-        <v>1080</v>
-      </c>
-      <c r="M36" s="1">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K36" s="1">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D37" s="6"/>
       <c r="H37" s="6"/>
       <c r="I37" s="1">
         <v>1</v>
       </c>
-      <c r="K37">
-        <v>0.5</v>
-      </c>
-      <c r="M37" s="1">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="K37" s="1">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D38" s="6"/>
+      <c r="F38" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="H38" s="6"/>
       <c r="I38" s="1">
-        <v>1</v>
-      </c>
-      <c r="K38">
-        <v>1</v>
-      </c>
-      <c r="M38" s="1">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="J38" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="K38" s="1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="D39" s="6"/>
-      <c r="F39" s="1" t="s">
-        <v>79</v>
-      </c>
       <c r="H39" s="6"/>
-      <c r="I39" s="1">
-        <v>3</v>
-      </c>
-      <c r="J39" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="K39">
-        <f t="shared" si="0"/>
-        <v>0.44999999999999996</v>
-      </c>
-      <c r="M39" s="1">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="D40" s="6"/>
       <c r="H40" s="6"/>
     </row>
-    <row r="41" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
-      <c r="D41" s="6"/>
+      <c r="C41" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>79</v>
+      </c>
       <c r="H41" s="6"/>
-      <c r="I41" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K41" s="1">
-        <f>SUM(K2:K40)</f>
-        <v>11.74954</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="D42" s="6"/>
       <c r="H42" s="6"/>
-      <c r="K42" s="6"/>
-    </row>
-    <row r="43" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="D43" s="6"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="K43" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="D44" s="6"/>
       <c r="H44" s="6"/>
-      <c r="K44" s="6"/>
-    </row>
-    <row r="45" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:11" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="D45" s="6"/>
       <c r="H45" s="6"/>
-      <c r="K45" s="6"/>
-    </row>
-    <row r="46" spans="1:14" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
+    </row>
+    <row r="46" spans="1:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="D46" s="6"/>
       <c r="H46" s="6"/>
-      <c r="K46" s="6"/>
-    </row>
-    <row r="47" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="D47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="K47" s="6"/>
-    </row>
-    <row r="48" spans="1:14" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="D48" s="7"/>
-      <c r="H48" s="7"/>
-      <c r="K48" s="7"/>
-    </row>
-    <row r="49" spans="3:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="D49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="K49" s="6"/>
-    </row>
-    <row r="50" spans="3:11" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:11" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="D47" s="7"/>
+      <c r="H47" s="7"/>
+    </row>
+    <row r="48" spans="1:11" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D48" s="6"/>
+      <c r="H48" s="6"/>
+    </row>
+    <row r="49" spans="3:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C49" s="1"/>
+    </row>
+    <row r="50" spans="3:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C50" s="1"/>
-      <c r="K50" s="8"/>
-    </row>
-    <row r="51" spans="3:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:11" ht="12.5" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="51" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="3:3" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="65" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="66" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="67" ht="12.5" x14ac:dyDescent="0.25"/>
@@ -2907,12 +2619,11 @@
     <row r="980" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="981" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="982" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="12.5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H12" r:id="rId1" xr:uid="{DA51463D-7099-4480-92F3-AC41DE28C746}"/>
-    <hyperlink ref="H21" r:id="rId2" xr:uid="{C55C3F2E-4DB8-4761-8AA8-AC5EB1EE0D71}"/>
+    <hyperlink ref="H11" r:id="rId1" xr:uid="{DA51463D-7099-4480-92F3-AC41DE28C746}"/>
+    <hyperlink ref="H20" r:id="rId2" xr:uid="{C55C3F2E-4DB8-4761-8AA8-AC5EB1EE0D71}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>